<commit_message>
feat: verify epic releases and complete stage 3 acceptance checks
</commit_message>
<xml_diff>
--- a/app/templates/credit_report.xlsx
+++ b/app/templates/credit_report.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Портфель" sheetId="1" r:id="R79eabf87fe2342b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Данные" sheetId="2" r:id="R54f202fd08a44332"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Портфель" sheetId="1" r:id="R1d3498d92cca42ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Данные" sheetId="2" r:id="Rd3bad51f171c4548"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Качество данных" sheetId="3" r:id="R1f83a662acd34da3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1432,4 +1433,625 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>Контроль покрытия источников. Независимый Python Decimal-эталон.</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="2"/>
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>Месяц</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Product ID</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>Регион</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>Строк месяца</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Кредитов на конец</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Нет снимка, кредиты</x:v>
+      </x:c>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>2026-01</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="2"/>
+      <x:c r="H5" s="2"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>2026-01</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="2"/>
+      <x:c r="H6" s="2"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>2026-01</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="2"/>
+      <x:c r="H7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>2026-01</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="2"/>
+      <x:c r="H8" s="2"/>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="n">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" s="2"/>
+      <x:c r="H9" s="2"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="2"/>
+      <x:c r="H10" s="2"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="2" t="str">
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="2"/>
+      <x:c r="H11" s="2"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="2"/>
+      <x:c r="H12" s="2"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="2" t="str">
+        <x:v>2026-03</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G13" s="2"/>
+      <x:c r="H13" s="2"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="2" t="str">
+        <x:v>2026-03</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G14" s="2"/>
+      <x:c r="H14" s="2"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="2" t="str">
+        <x:v>2026-03</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="2"/>
+      <x:c r="H15" s="2"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="2" t="str">
+        <x:v>2026-03</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="2"/>
+      <x:c r="H16" s="2"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="2" t="str">
+        <x:v>2026-04</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="n">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G17" s="2"/>
+      <x:c r="H17" s="2"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>2026-04</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="2"/>
+      <x:c r="H18" s="2"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>2026-04</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="2"/>
+      <x:c r="H19" s="2"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>2026-04</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="2"/>
+      <x:c r="H20" s="2"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>2026-05</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G21" s="2"/>
+      <x:c r="H21" s="2"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>2026-05</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G22" s="2"/>
+      <x:c r="H22" s="2"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="2" t="str">
+        <x:v>2026-05</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G23" s="2"/>
+      <x:c r="H23" s="2"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="2" t="str">
+        <x:v>2026-05</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F24" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="2"/>
+      <x:c r="H24" s="2"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="2" t="str">
+        <x:v>2026-06</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="n">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G25" s="2"/>
+      <x:c r="H25" s="2"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="2" t="str">
+        <x:v>2026-06</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="2"/>
+      <x:c r="H26" s="2"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="2" t="str">
+        <x:v>2026-06</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" s="2"/>
+      <x:c r="H27" s="2"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>2026-06</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F28" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" s="2"/>
+      <x:c r="H28" s="2"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="2"/>
+      <x:c r="B29" s="2"/>
+      <x:c r="C29" s="2"/>
+      <x:c r="D29" s="2"/>
+      <x:c r="E29" s="2"/>
+      <x:c r="F29" s="2"/>
+      <x:c r="G29" s="2"/>
+      <x:c r="H29" s="2"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="2"/>
+      <x:c r="B30" s="2"/>
+      <x:c r="C30" s="2"/>
+      <x:c r="D30" s="2"/>
+      <x:c r="E30" s="2"/>
+      <x:c r="F30" s="2"/>
+      <x:c r="G30" s="2"/>
+      <x:c r="H30" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>